<commit_message>
updated OR for autism with highlight
</commit_message>
<xml_diff>
--- a/parent_survey/ParentSurvey.xlsx
+++ b/parent_survey/ParentSurvey.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3c3887684911ee4/substack/autism/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stk\Documents\GitHub\autism\parent_survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="325" documentId="8_{CC3D48AD-5ABB-433F-A3EB-259011ADFC26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C2BA383-9019-43B1-BFFF-5D901115C0D7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826D76C6-09B2-45CB-A3C1-2E54506F8267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D736E639-7FA5-4501-9323-E7325C1F9870}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{D736E639-7FA5-4501-9323-E7325C1F9870}"/>
   </bookViews>
   <sheets>
     <sheet name="full OR analysis" sheetId="3" r:id="rId1"/>
@@ -160,9 +160,6 @@
     <t>SIDS</t>
   </si>
   <si>
-    <t>odds ratios for each symptom</t>
-  </si>
-  <si>
     <t>raw counts</t>
   </si>
   <si>
@@ -300,6 +297,9 @@
   <si>
     <t>Fact checkers should call me by phone if you want to fact check this. I have the contact info for each parent who filled out the form and the child's name who was being reported.</t>
   </si>
+  <si>
+    <t>odds for each symptom</t>
+  </si>
 </sst>
 </file>
 
@@ -308,7 +308,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,6 +328,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -353,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -371,6 +379,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,9 +401,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -429,7 +441,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -535,7 +547,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -677,7 +689,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -686,18 +698,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26CBD0F9-4E44-4D3D-B392-DBF33E18CFE9}">
   <dimension ref="A1:CO126"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="45.140625" customWidth="1"/>
-    <col min="14" max="14" width="8.85546875" style="3"/>
-    <col min="19" max="19" width="8.85546875" style="3"/>
-    <col min="24" max="24" width="8.85546875" style="3"/>
-    <col min="91" max="91" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="45.15625" customWidth="1"/>
+    <col min="14" max="14" width="8.83984375" style="3"/>
+    <col min="19" max="19" width="8.83984375" style="3"/>
+    <col min="24" max="24" width="8.83984375" style="3"/>
+    <col min="91" max="91" width="11.68359375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -935,37 +947,37 @@
         <v>101</v>
       </c>
       <c r="CD1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>60</v>
+      </c>
+      <c r="CF1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>62</v>
+      </c>
+      <c r="CH1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>64</v>
+      </c>
+      <c r="CJ1" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="CE1" t="s">
-        <v>61</v>
-      </c>
-      <c r="CF1" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="CG1" t="s">
-        <v>63</v>
-      </c>
-      <c r="CH1" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="CI1" t="s">
-        <v>65</v>
-      </c>
-      <c r="CJ1" s="5" t="s">
+      <c r="CK1" t="s">
         <v>67</v>
       </c>
-      <c r="CK1" t="s">
-        <v>68</v>
-      </c>
       <c r="CM1" t="s">
+        <v>75</v>
+      </c>
+      <c r="CO1" t="s">
         <v>76</v>
       </c>
-      <c r="CO1" t="s">
-        <v>77</v>
-      </c>
     </row>
-    <row r="2" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1231,7 +1243,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="3" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1391,7 +1403,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1643,7 +1655,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="5" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1897,7 +1909,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="6" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2141,239 +2153,239 @@
         <v>198</v>
       </c>
     </row>
-    <row r="7" spans="1:93" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:93" s="3" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>11</v>
       </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2">
         <v>26</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>6</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="2">
         <v>8</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="2">
         <v>9</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>8</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="2">
         <v>9</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>22</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>13</v>
       </c>
-      <c r="L7" s="1">
+      <c r="L7" s="2">
         <v>27</v>
       </c>
-      <c r="M7" s="1">
+      <c r="M7" s="2">
         <v>16</v>
       </c>
       <c r="N7" s="2">
         <v>47</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>3</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>29</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>3</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>5</v>
       </c>
       <c r="S7" s="2">
         <v>44</v>
       </c>
-      <c r="T7" s="1">
+      <c r="T7" s="2">
         <v>11</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>3</v>
       </c>
-      <c r="V7" s="1">
+      <c r="V7" s="2">
         <v>11</v>
       </c>
-      <c r="W7" s="1">
+      <c r="W7" s="2">
         <v>1</v>
       </c>
       <c r="X7" s="2">
         <v>53</v>
       </c>
-      <c r="Y7" s="1">
+      <c r="Y7" s="2">
         <v>6</v>
       </c>
-      <c r="Z7" s="1">
+      <c r="Z7" s="2">
         <v>8</v>
       </c>
-      <c r="AA7" s="1">
+      <c r="AA7" s="2">
         <v>4</v>
       </c>
-      <c r="AB7" s="1">
+      <c r="AB7" s="2">
         <v>6</v>
       </c>
-      <c r="AC7" s="1">
+      <c r="AC7" s="2">
         <v>24</v>
       </c>
-      <c r="AD7" s="1">
+      <c r="AD7" s="2">
         <v>5</v>
       </c>
-      <c r="AE7" s="1">
+      <c r="AE7" s="2">
         <v>2</v>
       </c>
-      <c r="AF7" s="1">
+      <c r="AF7" s="2">
         <v>4</v>
       </c>
-      <c r="AG7" s="1">
+      <c r="AG7" s="2">
         <v>3</v>
       </c>
-      <c r="AH7" s="1">
+      <c r="AH7" s="2">
         <v>27</v>
       </c>
-      <c r="AI7" s="1">
+      <c r="AI7" s="2">
         <v>2</v>
       </c>
-      <c r="AJ7" s="1">
+      <c r="AJ7" s="2">
         <v>3</v>
       </c>
-      <c r="AK7" s="1">
+      <c r="AK7" s="2">
         <v>3</v>
       </c>
-      <c r="AL7" s="1">
+      <c r="AL7" s="2">
         <v>2</v>
       </c>
-      <c r="AM7" s="1">
+      <c r="AM7" s="2">
         <v>6</v>
       </c>
-      <c r="AN7" s="1">
+      <c r="AN7" s="2">
         <v>2</v>
       </c>
-      <c r="AO7" s="1"/>
-      <c r="AP7" s="1">
-        <v>1</v>
-      </c>
-      <c r="AQ7" s="1">
+      <c r="AO7" s="2"/>
+      <c r="AP7" s="2">
+        <v>1</v>
+      </c>
+      <c r="AQ7" s="2">
         <v>2</v>
       </c>
-      <c r="AR7" s="1">
+      <c r="AR7" s="2">
         <v>8</v>
       </c>
-      <c r="AS7" s="1"/>
-      <c r="AT7" s="1">
-        <v>1</v>
-      </c>
-      <c r="AU7" s="1"/>
-      <c r="AV7" s="1">
-        <v>1</v>
-      </c>
-      <c r="AW7" s="1">
+      <c r="AS7" s="2"/>
+      <c r="AT7" s="2">
+        <v>1</v>
+      </c>
+      <c r="AU7" s="2"/>
+      <c r="AV7" s="2">
+        <v>1</v>
+      </c>
+      <c r="AW7" s="2">
         <v>2</v>
       </c>
-      <c r="AX7" s="1"/>
-      <c r="AY7" s="1"/>
-      <c r="AZ7" s="1">
-        <v>1</v>
-      </c>
-      <c r="BA7" s="1"/>
-      <c r="BB7" s="1">
+      <c r="AX7" s="2"/>
+      <c r="AY7" s="2"/>
+      <c r="AZ7" s="2">
+        <v>1</v>
+      </c>
+      <c r="BA7" s="2"/>
+      <c r="BB7" s="2">
         <v>7</v>
       </c>
-      <c r="BC7" s="1"/>
-      <c r="BD7" s="1"/>
-      <c r="BE7" s="1"/>
-      <c r="BF7" s="1">
+      <c r="BC7" s="2"/>
+      <c r="BD7" s="2"/>
+      <c r="BE7" s="2"/>
+      <c r="BF7" s="2">
         <v>2</v>
       </c>
-      <c r="BG7" s="1"/>
-      <c r="BH7" s="1"/>
-      <c r="BI7" s="1"/>
-      <c r="BJ7" s="1">
-        <v>1</v>
-      </c>
-      <c r="BK7" s="1"/>
-      <c r="BL7" s="1"/>
-      <c r="BM7" s="1"/>
-      <c r="BN7" s="1">
-        <v>1</v>
-      </c>
-      <c r="BO7" s="1"/>
-      <c r="BP7" s="1">
-        <v>1</v>
-      </c>
-      <c r="BQ7" s="1"/>
-      <c r="BR7" s="1"/>
-      <c r="BS7" s="1"/>
-      <c r="BT7" s="1">
-        <v>1</v>
-      </c>
-      <c r="BU7" s="1"/>
-      <c r="BV7" s="1">
-        <v>1</v>
-      </c>
-      <c r="BW7" s="1"/>
-      <c r="BX7" s="1"/>
-      <c r="BY7" s="1"/>
-      <c r="BZ7" s="1"/>
-      <c r="CA7" s="1">
-        <v>1</v>
-      </c>
-      <c r="CB7" s="1">
-        <v>1</v>
-      </c>
-      <c r="CD7">
+      <c r="BG7" s="2"/>
+      <c r="BH7" s="2"/>
+      <c r="BI7" s="2"/>
+      <c r="BJ7" s="2">
+        <v>1</v>
+      </c>
+      <c r="BK7" s="2"/>
+      <c r="BL7" s="2"/>
+      <c r="BM7" s="2"/>
+      <c r="BN7" s="2">
+        <v>1</v>
+      </c>
+      <c r="BO7" s="2"/>
+      <c r="BP7" s="2">
+        <v>1</v>
+      </c>
+      <c r="BQ7" s="2"/>
+      <c r="BR7" s="2"/>
+      <c r="BS7" s="2"/>
+      <c r="BT7" s="2">
+        <v>1</v>
+      </c>
+      <c r="BU7" s="2"/>
+      <c r="BV7" s="2">
+        <v>1</v>
+      </c>
+      <c r="BW7" s="2"/>
+      <c r="BX7" s="2"/>
+      <c r="BY7" s="2"/>
+      <c r="BZ7" s="2"/>
+      <c r="CA7" s="2">
+        <v>1</v>
+      </c>
+      <c r="CB7" s="2">
+        <v>1</v>
+      </c>
+      <c r="CD7" s="3">
         <f t="shared" si="7"/>
         <v>49</v>
       </c>
-      <c r="CE7">
+      <c r="CE7" s="3">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="CF7">
+      <c r="CF7" s="3">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
-      <c r="CG7">
+      <c r="CG7" s="3">
         <f t="shared" si="2"/>
         <v>48</v>
       </c>
-      <c r="CH7">
+      <c r="CH7" s="3">
         <f t="shared" si="3"/>
         <v>52</v>
       </c>
-      <c r="CI7">
+      <c r="CI7" s="3">
         <f t="shared" si="4"/>
         <v>71</v>
       </c>
-      <c r="CJ7">
+      <c r="CJ7" s="3">
         <f t="shared" si="5"/>
         <v>78</v>
       </c>
-      <c r="CK7">
+      <c r="CK7" s="3">
         <f t="shared" si="6"/>
         <v>103</v>
       </c>
-      <c r="CM7">
+      <c r="CM7" s="3">
         <f t="shared" si="8"/>
         <v>352</v>
       </c>
-      <c r="CO7">
+      <c r="CO7" s="3">
         <f t="shared" si="9"/>
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2599,7 +2611,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="9" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2801,7 +2813,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2945,7 +2957,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -3101,7 +3113,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -3293,7 +3305,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -3465,7 +3477,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -3653,7 +3665,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -3839,7 +3851,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -3993,7 +4005,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -4149,7 +4161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -4341,7 +4353,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -4587,7 +4599,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="20" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -4815,7 +4827,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="21" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -5003,7 +5015,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -5231,7 +5243,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -5469,7 +5481,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="24" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -5651,7 +5663,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -5837,7 +5849,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -6063,7 +6075,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -6303,7 +6315,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="28" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -6513,7 +6525,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -6697,7 +6709,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -6849,7 +6861,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
         <v>39</v>
       </c>
@@ -6976,7 +6988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="1" t="s">
         <v>29</v>
       </c>
@@ -7196,7 +7208,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1" t="s">
         <v>30</v>
       </c>
@@ -7396,7 +7408,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="34" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
         <v>31</v>
       </c>
@@ -7528,7 +7540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="1" t="s">
         <v>32</v>
       </c>
@@ -7670,7 +7682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="1" t="s">
         <v>33</v>
       </c>
@@ -7888,7 +7900,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="1" t="s">
         <v>34</v>
       </c>
@@ -8078,7 +8090,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="1" t="s">
         <v>35</v>
       </c>
@@ -8282,7 +8294,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="1" t="s">
         <v>36</v>
       </c>
@@ -8510,7 +8522,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="40" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="1" t="s">
         <v>37</v>
       </c>
@@ -8752,7 +8764,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="41" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="1" t="s">
         <v>38</v>
       </c>
@@ -9031,12 +9043,12 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="44" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="2" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="1" t="s">
         <v>0</v>
       </c>
@@ -9385,7 +9397,7 @@
         <v>1.2733900364520048</v>
       </c>
       <c r="CM46">
-        <f t="shared" ref="CM46:CO46" si="13">CM2/(CM$41-CM2)</f>
+        <f t="shared" ref="CM46" si="13">CM2/(CM$41-CM2)</f>
         <v>1.6336052202283851</v>
       </c>
       <c r="CO46">
@@ -9393,7 +9405,7 @@
         <v>0.81785392245266009</v>
       </c>
     </row>
-    <row r="47" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="1" t="s">
         <v>1</v>
       </c>
@@ -9750,7 +9762,7 @@
         <v>1.4903129657228018E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="1" t="s">
         <v>2</v>
       </c>
@@ -10107,7 +10119,7 @@
         <v>0.17277486910994763</v>
       </c>
     </row>
-    <row r="49" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="1" t="s">
         <v>3</v>
       </c>
@@ -10464,7 +10476,7 @@
         <v>0.26633165829145727</v>
       </c>
     </row>
-    <row r="50" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="1" t="s">
         <v>4</v>
       </c>
@@ -10821,11 +10833,11 @@
         <v>0.10891089108910891</v>
       </c>
     </row>
-    <row r="51" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="9">
         <f t="shared" ref="B51:BM51" si="31">B7/(B$41-B7)</f>
         <v>1.4416775884665793E-2</v>
       </c>
@@ -11178,7 +11190,7 @@
         <v>6.4976228209191758E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="1" t="s">
         <v>6</v>
       </c>
@@ -11535,7 +11547,7 @@
         <v>8.4454007530930603E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="1" t="s">
         <v>7</v>
       </c>
@@ -11892,7 +11904,7 @@
         <v>1.8181818181818181E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="1" t="s">
         <v>8</v>
       </c>
@@ -12249,7 +12261,7 @@
         <v>9.930486593843098E-4</v>
       </c>
     </row>
-    <row r="55" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="1" t="s">
         <v>9</v>
       </c>
@@ -12606,7 +12618,7 @@
         <v>3.9840637450199202E-3</v>
       </c>
     </row>
-    <row r="56" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="1" t="s">
         <v>10</v>
       </c>
@@ -12963,7 +12975,7 @@
         <v>1.6129032258064516E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="1" t="s">
         <v>11</v>
       </c>
@@ -13320,7 +13332,7 @@
         <v>9.5142714071106659E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="1" t="s">
         <v>12</v>
       </c>
@@ -13677,7 +13689,7 @@
         <v>2.3350253807106598E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="1" t="s">
         <v>13</v>
       </c>
@@ -14034,7 +14046,7 @@
         <v>4.4843049327354259E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="1" t="s">
         <v>14</v>
       </c>
@@ -14391,7 +14403,7 @@
         <v>1.9880715705765406E-3</v>
       </c>
     </row>
-    <row r="61" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="1" t="s">
         <v>15</v>
       </c>
@@ -14748,7 +14760,7 @@
         <v>4.9627791563275434E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="1" t="s">
         <v>16</v>
       </c>
@@ -15105,7 +15117,7 @@
         <v>1.6129032258064516E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="1" t="s">
         <v>17</v>
       </c>
@@ -15462,7 +15474,7 @@
         <v>0.11258278145695365</v>
       </c>
     </row>
-    <row r="64" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="1" t="s">
         <v>18</v>
       </c>
@@ -15819,7 +15831,7 @@
         <v>5.8823529411764705E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="1" t="s">
         <v>19</v>
       </c>
@@ -16176,7 +16188,7 @@
         <v>1.0526315789473684E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="1" t="s">
         <v>20</v>
       </c>
@@ -16533,7 +16545,7 @@
         <v>7.5200000000000003E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="1" t="s">
         <v>21</v>
       </c>
@@ -16890,7 +16902,7 @@
         <v>7.8074866310160432E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="1" t="s">
         <v>22</v>
       </c>
@@ -17247,7 +17259,7 @@
         <v>9.5142714071106659E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="1" t="s">
         <v>23</v>
       </c>
@@ -17604,7 +17616,7 @@
         <v>1.1033099297893681E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="1" t="s">
         <v>24</v>
       </c>
@@ -17961,7 +17973,7 @@
         <v>6.0494476591267755E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="1" t="s">
         <v>25</v>
       </c>
@@ -18318,7 +18330,7 @@
         <v>6.1611374407582936E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="1" t="s">
         <v>26</v>
       </c>
@@ -18675,7 +18687,7 @@
         <v>2.231237322515213E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="1" t="s">
         <v>27</v>
       </c>
@@ -19032,7 +19044,7 @@
         <v>5.4862842892768084E-3</v>
       </c>
     </row>
-    <row r="74" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="1" t="s">
         <v>28</v>
       </c>
@@ -19389,7 +19401,7 @@
         <v>5.9880239520958087E-3</v>
       </c>
     </row>
-    <row r="75" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="1" t="s">
         <v>39</v>
       </c>
@@ -19746,7 +19758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="1" t="s">
         <v>29</v>
       </c>
@@ -20103,7 +20115,7 @@
         <v>4.2399172699069287E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="1" t="s">
         <v>30</v>
       </c>
@@ -20460,7 +20472,7 @@
         <v>2.5954198473282442E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" s="1" t="s">
         <v>31</v>
       </c>
@@ -20817,7 +20829,7 @@
         <v>4.9627791563275434E-4</v>
       </c>
     </row>
-    <row r="79" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" s="1" t="s">
         <v>32</v>
       </c>
@@ -21174,7 +21186,7 @@
         <v>4.9627791563275434E-4</v>
       </c>
     </row>
-    <row r="80" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" s="1" t="s">
         <v>33</v>
       </c>
@@ -21531,7 +21543,7 @@
         <v>3.2786885245901641E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" s="1" t="s">
         <v>34</v>
       </c>
@@ -21888,7 +21900,7 @@
         <v>6.993006993006993E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" s="1" t="s">
         <v>35</v>
       </c>
@@ -22245,7 +22257,7 @@
         <v>2.0242914979757085E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" s="1" t="s">
         <v>36</v>
       </c>
@@ -22602,7 +22614,7 @@
         <v>6.9496021220159146E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" s="1" t="s">
         <v>37</v>
       </c>
@@ -22959,13 +22971,13 @@
         <v>7.0063694267515922E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:93" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:93" s="3" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="T87"/>
     </row>
-    <row r="88" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" s="1" t="s">
         <v>0</v>
       </c>
@@ -23318,7 +23330,7 @@
         <v>0.14858720117842222</v>
       </c>
     </row>
-    <row r="89" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" s="1" t="s">
         <v>1</v>
       </c>
@@ -23671,7 +23683,7 @@
         <v>0.38301043219076003</v>
       </c>
     </row>
-    <row r="90" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" s="1" t="s">
         <v>2</v>
       </c>
@@ -24024,7 +24036,7 @@
         <v>7.2565445026178006</v>
       </c>
     </row>
-    <row r="91" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" s="1" t="s">
         <v>3</v>
       </c>
@@ -24377,7 +24389,7 @@
         <v>7.6621569385388479</v>
       </c>
     </row>
-    <row r="92" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" s="1" t="s">
         <v>4</v>
       </c>
@@ -24730,360 +24742,360 @@
         <v>9.2574257425742577</v>
       </c>
     </row>
-    <row r="93" spans="1:93" x14ac:dyDescent="0.25">
-      <c r="A93" s="1" t="s">
+    <row r="93" spans="1:93" s="9" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A93" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D93">
+      <c r="D93" s="9">
         <f t="shared" ref="D93:BO93" si="187">IF($B51&gt;0, D51/$B51,"")</f>
         <v>1.5244755244755246</v>
       </c>
-      <c r="E93">
+      <c r="E93" s="9">
         <f t="shared" si="187"/>
         <v>2.2742175856929956</v>
       </c>
-      <c r="F93">
+      <c r="F93" s="9">
         <f t="shared" si="187"/>
         <v>2.9360269360269355</v>
       </c>
-      <c r="G93">
+      <c r="G93" s="9">
         <f t="shared" si="187"/>
         <v>2.0878686530860442</v>
       </c>
-      <c r="H93">
+      <c r="H93" s="9">
         <f t="shared" si="187"/>
         <v>2.1508104298801971</v>
       </c>
-      <c r="I93">
+      <c r="I93" s="9">
         <f t="shared" si="187"/>
         <v>1.6214876033057852</v>
       </c>
-      <c r="J93">
+      <c r="J93" s="9">
         <f t="shared" si="187"/>
         <v>2.9233716475095783</v>
       </c>
-      <c r="K93">
+      <c r="K93" s="9">
         <f t="shared" si="187"/>
         <v>3.6359970674486806</v>
       </c>
-      <c r="L93">
+      <c r="L93" s="9">
         <f t="shared" si="187"/>
         <v>4.0189231369488878</v>
       </c>
-      <c r="M93">
+      <c r="M93" s="9">
         <f t="shared" si="187"/>
         <v>5.0909090909090908</v>
       </c>
-      <c r="N93" s="3">
+      <c r="N93" s="9">
         <f t="shared" si="187"/>
         <v>3.8996302740321878</v>
       </c>
-      <c r="O93">
+      <c r="O93" s="9">
         <f t="shared" si="187"/>
         <v>2.6340621403912543</v>
       </c>
-      <c r="P93">
+      <c r="P93" s="9">
         <f t="shared" si="187"/>
         <v>3.4622124863088715</v>
       </c>
-      <c r="Q93">
+      <c r="Q93" s="9">
         <f t="shared" si="187"/>
         <v>2.0401069518716577</v>
       </c>
-      <c r="R93">
+      <c r="R93" s="9">
         <f t="shared" si="187"/>
         <v>2.7969208211143695</v>
       </c>
-      <c r="S93" s="3">
+      <c r="S93" s="9">
         <f t="shared" si="187"/>
         <v>4.1751025991792066</v>
       </c>
-      <c r="T93">
+      <c r="T93" s="9">
         <f t="shared" si="187"/>
         <v>6.3583333333333325</v>
       </c>
-      <c r="U93">
+      <c r="U93" s="9">
         <f t="shared" si="187"/>
         <v>2.2867132867132867</v>
       </c>
-      <c r="V93">
+      <c r="V93" s="9">
         <f t="shared" si="187"/>
         <v>4.7987421383647799</v>
       </c>
-      <c r="W93">
+      <c r="W93" s="9">
         <f t="shared" si="187"/>
         <v>2.0401069518716577</v>
       </c>
-      <c r="X93" s="3">
+      <c r="X93" s="9">
         <f t="shared" si="187"/>
         <v>4.8499640201487164</v>
       </c>
-      <c r="Y93">
+      <c r="Y93" s="9">
         <f t="shared" si="187"/>
         <v>9.9090909090909083</v>
       </c>
-      <c r="Z93">
+      <c r="Z93" s="9">
         <f t="shared" si="187"/>
         <v>9.735247208931419</v>
       </c>
-      <c r="AA93">
+      <c r="AA93" s="9">
         <f t="shared" si="187"/>
         <v>4.268531468531469</v>
       </c>
-      <c r="AB93">
+      <c r="AB93" s="9">
         <f t="shared" si="187"/>
         <v>4.8962566844919779</v>
       </c>
-      <c r="AC93">
+      <c r="AC93" s="9">
         <f t="shared" si="187"/>
         <v>4.7699921854649645</v>
       </c>
-      <c r="AD93">
+      <c r="AD93" s="9">
         <f t="shared" si="187"/>
         <v>7.0779220779220777</v>
       </c>
-      <c r="AE93">
+      <c r="AE93" s="9">
         <f t="shared" si="187"/>
         <v>3.4681818181818183</v>
       </c>
-      <c r="AF93">
+      <c r="AF93" s="9">
         <f t="shared" si="187"/>
         <v>4.9545454545454541</v>
       </c>
-      <c r="AG93">
+      <c r="AG93" s="9">
         <f t="shared" si="187"/>
         <v>8.3236363636363624</v>
       </c>
-      <c r="AH93">
+      <c r="AH93" s="9">
         <f t="shared" si="187"/>
         <v>5.4442389006342493</v>
       </c>
-      <c r="AI93">
+      <c r="AI93" s="9">
         <f t="shared" si="187"/>
         <v>5.1380471380471375</v>
       </c>
-      <c r="AJ93">
+      <c r="AJ93" s="9">
         <f t="shared" si="187"/>
         <v>4.624242424242424</v>
       </c>
-      <c r="AK93">
+      <c r="AK93" s="9">
         <f t="shared" si="187"/>
         <v>6.7126099706744862</v>
       </c>
-      <c r="AL93">
+      <c r="AL93" s="9">
         <f t="shared" si="187"/>
         <v>5.5490909090909089</v>
       </c>
-      <c r="AM93">
+      <c r="AM93" s="9">
         <f t="shared" si="187"/>
         <v>4.0406001765225064</v>
       </c>
-      <c r="AN93">
+      <c r="AN93" s="9">
         <f t="shared" si="187"/>
         <v>4.9545454545454541</v>
       </c>
-      <c r="AO93">
+      <c r="AO93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="AP93">
+      <c r="AP93" s="9">
         <f t="shared" si="187"/>
         <v>3.0158102766798418</v>
       </c>
-      <c r="AQ93">
+      <c r="AQ93" s="9">
         <f t="shared" si="187"/>
         <v>8.670454545454545</v>
       </c>
-      <c r="AR93">
+      <c r="AR93" s="9">
         <f t="shared" si="187"/>
         <v>3.8804831532104256</v>
       </c>
-      <c r="AS93">
+      <c r="AS93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="AT93">
+      <c r="AT93" s="9">
         <f t="shared" si="187"/>
         <v>8.670454545454545</v>
       </c>
-      <c r="AU93">
+      <c r="AU93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="AV93">
+      <c r="AV93" s="9">
         <f t="shared" si="187"/>
         <v>9.9090909090909083</v>
       </c>
-      <c r="AW93">
+      <c r="AW93" s="9">
         <f t="shared" si="187"/>
         <v>4.3352272727272725</v>
       </c>
-      <c r="AX93">
+      <c r="AX93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="AY93">
+      <c r="AY93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="AZ93">
+      <c r="AZ93" s="9">
         <f t="shared" si="187"/>
         <v>7.7070707070707067</v>
       </c>
-      <c r="BA93">
+      <c r="BA93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BB93">
+      <c r="BB93" s="9">
         <f t="shared" si="187"/>
         <v>4.9044995408631769</v>
       </c>
-      <c r="BC93">
+      <c r="BC93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BD93">
+      <c r="BD93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BE93">
+      <c r="BE93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BF93">
+      <c r="BF93" s="9">
         <f t="shared" si="187"/>
         <v>27.745454545454546</v>
       </c>
-      <c r="BG93">
+      <c r="BG93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BH93">
+      <c r="BH93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BI93">
+      <c r="BI93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BJ93">
+      <c r="BJ93" s="9">
         <f t="shared" si="187"/>
         <v>1.6515151515151514</v>
       </c>
-      <c r="BK93">
+      <c r="BK93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BL93">
+      <c r="BL93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BM93">
+      <c r="BM93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BN93">
+      <c r="BN93" s="9">
         <f t="shared" si="187"/>
         <v>6.3057851239669418</v>
       </c>
-      <c r="BO93">
+      <c r="BO93" s="9">
         <f t="shared" si="187"/>
         <v>0</v>
       </c>
-      <c r="BP93">
+      <c r="BP93" s="9">
         <f t="shared" ref="BP93:CB93" si="188">IF($B51&gt;0, BP51/$B51,"")</f>
         <v>4.9545454545454541</v>
       </c>
-      <c r="BQ93">
+      <c r="BQ93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BR93">
+      <c r="BR93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BS93">
+      <c r="BS93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BT93">
+      <c r="BT93" s="9">
         <f t="shared" si="188"/>
         <v>69.36363636363636</v>
       </c>
-      <c r="BU93">
+      <c r="BU93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BV93">
+      <c r="BV93" s="9">
         <f t="shared" si="188"/>
         <v>9.9090909090909083</v>
       </c>
-      <c r="BW93">
+      <c r="BW93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BX93">
+      <c r="BX93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BY93">
+      <c r="BY93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="BZ93">
+      <c r="BZ93" s="9">
         <f t="shared" si="188"/>
         <v>0</v>
       </c>
-      <c r="CA93">
+      <c r="CA93" s="9">
         <f t="shared" si="188"/>
         <v>13.872727272727273</v>
       </c>
-      <c r="CB93">
+      <c r="CB93" s="9">
         <f t="shared" si="188"/>
         <v>8.670454545454545</v>
       </c>
-      <c r="CD93">
+      <c r="CD93" s="9">
         <f t="shared" ref="CD93:CK93" si="189">IF($B51&gt;0, CD51/$B51,"")</f>
         <v>1.8332352652741002</v>
       </c>
-      <c r="CE93">
+      <c r="CE93" s="9">
         <f t="shared" si="189"/>
         <v>2.3146100401213423</v>
       </c>
-      <c r="CF93">
+      <c r="CF93" s="9">
         <f t="shared" si="189"/>
         <v>2.0852021541676713</v>
       </c>
-      <c r="CG93">
+      <c r="CG93" s="9">
         <f t="shared" si="189"/>
         <v>2.2742175856929956</v>
       </c>
-      <c r="CH93">
+      <c r="CH93" s="9">
         <f t="shared" si="189"/>
         <v>2.5526603615775594</v>
       </c>
-      <c r="CI93">
+      <c r="CI93" s="9">
         <f t="shared" si="189"/>
         <v>3.0381358308563735</v>
       </c>
-      <c r="CJ93">
+      <c r="CJ93" s="9">
         <f t="shared" si="189"/>
         <v>3.7210203826434913</v>
       </c>
-      <c r="CK93">
+      <c r="CK93" s="9">
         <f t="shared" si="189"/>
         <v>4.0409810777457835</v>
       </c>
-      <c r="CM93">
+      <c r="CM93" s="9">
         <f t="shared" ref="CM93:CO93" si="190">IF($B51&gt;0, CM51/$B51,"")</f>
         <v>3.1626943005181345</v>
       </c>
-      <c r="CO93">
+      <c r="CO93" s="9">
         <f t="shared" si="190"/>
         <v>4.5069874657830278</v>
       </c>
     </row>
-    <row r="94" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" s="1" t="s">
         <v>6</v>
       </c>
@@ -25436,7 +25448,7 @@
         <v>21.704679935449164</v>
       </c>
     </row>
-    <row r="95" spans="1:93" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:93" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" s="7" t="s">
         <v>7</v>
       </c>
@@ -25789,7 +25801,7 @@
         <v>0.91999999999999993</v>
       </c>
     </row>
-    <row r="96" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" s="1" t="s">
         <v>8</v>
       </c>
@@ -26142,7 +26154,7 @@
         <v>0.76762661370407137</v>
       </c>
     </row>
-    <row r="97" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" s="1" t="s">
         <v>9</v>
       </c>
@@ -26495,7 +26507,7 @@
         <v>3.0796812749003979</v>
       </c>
     </row>
-    <row r="98" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A98" s="1" t="s">
         <v>10</v>
       </c>
@@ -26848,7 +26860,7 @@
         <v>4.1451612903225801</v>
       </c>
     </row>
-    <row r="99" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A99" s="1" t="s">
         <v>11</v>
       </c>
@@ -27201,7 +27213,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A100" s="1" t="s">
         <v>12</v>
       </c>
@@ -27554,7 +27566,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A101" s="1" t="s">
         <v>13</v>
       </c>
@@ -27907,7 +27919,7 @@
         <v>3.4663677130044839</v>
       </c>
     </row>
-    <row r="102" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A102" s="1" t="s">
         <v>14</v>
       </c>
@@ -28260,7 +28272,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A103" s="1" t="s">
         <v>15</v>
       </c>
@@ -28613,7 +28625,7 @@
         <v>0.19156327543424317</v>
       </c>
     </row>
-    <row r="104" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A104" s="1" t="s">
         <v>16</v>
       </c>
@@ -28966,7 +28978,7 @@
         <v>4.1451612903225801</v>
       </c>
     </row>
-    <row r="105" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" s="1" t="s">
         <v>17</v>
       </c>
@@ -29319,7 +29331,7 @@
         <v>3.3729801324503317</v>
       </c>
     </row>
-    <row r="106" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A106" s="1" t="s">
         <v>18</v>
       </c>
@@ -29672,7 +29684,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A107" s="1" t="s">
         <v>19</v>
       </c>
@@ -30025,7 +30037,7 @@
         <v>1.0078947368421052</v>
       </c>
     </row>
-    <row r="108" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A108" s="1" t="s">
         <v>20</v>
       </c>
@@ -30378,7 +30390,7 @@
         <v>1.6367058823529412</v>
       </c>
     </row>
-    <row r="109" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A109" s="1" t="s">
         <v>21</v>
       </c>
@@ -30731,7 +30743,7 @@
         <v>5.4155566358774916</v>
       </c>
     </row>
-    <row r="110" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A110" s="1" t="s">
         <v>22</v>
       </c>
@@ -31084,7 +31096,7 @@
         <v>3.6725087631447169</v>
       </c>
     </row>
-    <row r="111" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A111" s="1" t="s">
         <v>23</v>
       </c>
@@ -31437,7 +31449,7 @@
         <v>2.8355065195586762</v>
       </c>
     </row>
-    <row r="112" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A112" s="1" t="s">
         <v>24</v>
       </c>
@@ -31790,7 +31802,7 @@
         <v>6.628466220786053</v>
       </c>
     </row>
-    <row r="113" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" s="1" t="s">
         <v>25</v>
       </c>
@@ -32143,7 +32155,7 @@
         <v>6.7508463100880167</v>
       </c>
     </row>
-    <row r="114" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A114" s="1" t="s">
         <v>26</v>
       </c>
@@ -32496,7 +32508,7 @@
         <v>4.2951318458417846</v>
       </c>
     </row>
-    <row r="115" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A115" s="1" t="s">
         <v>27</v>
       </c>
@@ -32849,7 +32861,7 @@
         <v>2.1177057356608477</v>
       </c>
     </row>
-    <row r="116" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A116" s="1" t="s">
         <v>28</v>
       </c>
@@ -33202,7 +33214,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A117" s="1" t="s">
         <v>39</v>
       </c>
@@ -33555,7 +33567,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A118" s="1" t="s">
         <v>29</v>
       </c>
@@ -33908,7 +33920,7 @@
         <v>32.774560496380559</v>
       </c>
     </row>
-    <row r="119" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A119" s="1" t="s">
         <v>30</v>
       </c>
@@ -34261,7 +34273,7 @@
         <v>3.9917557251908398</v>
       </c>
     </row>
-    <row r="120" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A120" s="1" t="s">
         <v>31</v>
       </c>
@@ -34614,7 +34626,7 @@
         <v>7.632754342431762E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A121" s="1" t="s">
         <v>32</v>
       </c>
@@ -34967,7 +34979,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" s="1" t="s">
         <v>33</v>
       </c>
@@ -35320,7 +35332,7 @@
         <v>5.0426229508196725</v>
       </c>
     </row>
-    <row r="123" spans="1:93" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A123" s="1" t="s">
         <v>34</v>
       </c>
@@ -35673,7 +35685,7 @@
         <v>2.6993006993006992</v>
       </c>
     </row>
-    <row r="124" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A124" s="1" t="s">
         <v>35</v>
       </c>
@@ -36026,7 +36038,7 @@
         <v>5.2024291497975712</v>
       </c>
     </row>
-    <row r="125" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:93" x14ac:dyDescent="0.55000000000000004">
       <c r="A125" s="1" t="s">
         <v>36</v>
       </c>
@@ -36379,7 +36391,7 @@
         <v>4.4129973474801059</v>
       </c>
     </row>
-    <row r="126" spans="1:93" ht="30" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:93" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A126" s="1" t="s">
         <v>37</v>
       </c>
@@ -36744,13 +36756,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43A54107-0296-409E-9597-115ADC7C760C}">
   <dimension ref="A1:B33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.68359375" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -36758,7 +36770,7 @@
         <v>7.2565445026178006</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -36766,7 +36778,7 @@
         <v>7.6621569385388479</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -36774,7 +36786,7 @@
         <v>9.2574257425742577</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -36782,7 +36794,7 @@
         <v>4.5069874657830278</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -36790,15 +36802,15 @@
         <v>21.704679935449164</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B6" s="8">
         <v>0.91999999999999993</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -36806,7 +36818,7 @@
         <v>0.76762661370407137</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -36814,7 +36826,7 @@
         <v>3.0796812749003979</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -36822,7 +36834,7 @@
         <v>4.1451612903225801</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -36830,7 +36842,7 @@
         <v>3.4663677130044839</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -36838,7 +36850,7 @@
         <v>4.1451612903225801</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -36846,7 +36858,7 @@
         <v>3.3729801324503317</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -36854,7 +36866,7 @@
         <v>1.0078947368421052</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -36862,7 +36874,7 @@
         <v>1.6367058823529412</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -36870,7 +36882,7 @@
         <v>5.4155566358774916</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -36878,7 +36890,7 @@
         <v>3.6725087631447169</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -36886,7 +36898,7 @@
         <v>2.8355065195586762</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -36894,7 +36906,7 @@
         <v>6.628466220786053</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -36902,7 +36914,7 @@
         <v>6.7508463100880167</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -36910,7 +36922,7 @@
         <v>4.2951318458417846</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -36918,7 +36930,7 @@
         <v>2.1177057356608477</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="1" t="s">
         <v>29</v>
       </c>
@@ -36926,7 +36938,7 @@
         <v>32.774560496380559</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="1" t="s">
         <v>30</v>
       </c>
@@ -36934,7 +36946,7 @@
         <v>3.9917557251908398</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -36942,7 +36954,7 @@
         <v>5.0426229508196725</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
@@ -36950,7 +36962,7 @@
         <v>2.6993006993006992</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
@@ -36958,7 +36970,7 @@
         <v>5.2024291497975712</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
         <v>36</v>
       </c>
@@ -36966,7 +36978,7 @@
         <v>4.4129973474801059</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
@@ -36974,14 +36986,14 @@
         <v>8.968152866242038</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" t="s">
         <v>79</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -36993,170 +37005,170 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94490590-B041-44AF-9DC2-70CFB89FC8C0}">
   <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>82</v>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="4" t="s">
+        <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="4"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="4"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="4"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>69</v>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>70</v>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>71</v>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>72</v>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" t="s">
+        <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>73</v>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>74</v>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" t="s">
+        <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>60</v>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>53</v>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>48</v>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" t="s">
+        <v>57</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>